<commit_message>
feat: engine v2 — historical EM anchoring, concordance gate, WACC floor + re-renders
Engine changes (fmp_3statementv6.py + report_bridge.py):
- Rule 21: Historical EV/EBITDA anchoring (5yr avg × 0.80, capped 28×, floored at quality-premium base)
- Rule 16: Valuation concordance gate — premium/discount verdict override when both GG + EM agree
- Rule 11: WACC floor 8.5%
- Rule 15: Rescale suppression on data-fetch gaps
- Score audit script extended with full valuation field diff

Dashboard: removed stale WIP banner

Re-rendered 22 tickers against updated engine:
AAPL ABBV ADBE AMD BAC COST CVX C DIS FDX F INTC JNJ JPM KO NKE NVDA PEP SNAP SOFI V WMT

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/CVX_model.xlsx
+++ b/static/excel/CVX_model.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Ratios &amp; FCF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Segments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WACC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DCF" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Scorecard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios &amp; FCF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7339,11 +7339,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>371632.56</v>
+        <v>381251.988</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $186.6</t>
+          <t>FMP marketCap  |  price $191.43</t>
         </is>
       </c>
     </row>
@@ -7425,11 +7425,11 @@
         </is>
       </c>
       <c r="B12" s="46" t="n">
-        <v>0.0446</v>
+        <v>0.0457</v>
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-13</t>
+          <t>FRED series DGS10  |  latest: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="B13" s="48" t="n">
-        <v>0.0446</v>
+        <v>0.0457</v>
       </c>
       <c r="C13" s="49" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="B19" s="50" t="n">
-        <v>0.836</v>
+        <v>0.834</v>
       </c>
       <c r="C19" s="44">
         <f> unlevered × (1 + (1 − t) × D/E)</f>
@@ -7526,7 +7526,7 @@
         </is>
       </c>
       <c r="B20" s="51" t="n">
-        <v>0.668</v>
+        <v>0.667</v>
       </c>
       <c r="C20" s="49" t="inlineStr">
         <is>
@@ -7700,11 +7700,11 @@
         </is>
       </c>
       <c r="B35" s="46" t="n">
-        <v>0.05</v>
+        <v>0.05110000000000001</v>
       </c>
       <c r="C35" s="44" t="inlineStr">
         <is>
-          <t>Rf 4.46% + spread 0.54%</t>
+          <t>Rf 4.57% + spread 0.54%</t>
         </is>
       </c>
     </row>
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="B37" s="48" t="n">
-        <v>0.0435</v>
+        <v>0.044</v>
       </c>
       <c r="C37" s="49" t="inlineStr">
         <is>
@@ -7795,16 +7795,16 @@
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="54" t="inlineStr">
         <is>
-          <t>WACC  =  (E/V × Re)  +  (D/V × Rd × (1 − t))</t>
+          <t>WACC  =  MAX(8.5%, (E/V × Re) + (D/V × Rd × (1 − t)))</t>
         </is>
       </c>
       <c r="B44" s="55">
-        <f>B8*B28+B9*B37*(1-B41)</f>
+        <f>MAX(0.085, B8*B28+B9*B37*(1-B41))</f>
         <v/>
       </c>
       <c r="C44" s="56" t="inlineStr">
         <is>
-          <t>Used as discount rate in DCF tab</t>
+          <t>Floored 8.5% (D-001); raw formula below</t>
         </is>
       </c>
     </row>
@@ -8167,13 +8167,13 @@
         <v/>
       </c>
       <c r="G7" s="71" t="n">
-        <v>0.2289</v>
+        <v>0.239</v>
       </c>
       <c r="H7" s="71" t="n">
-        <v>-0.1034</v>
+        <v>-0.1166</v>
       </c>
       <c r="I7" s="71" t="n">
-        <v>-0.0009</v>
+        <v>-0.0015</v>
       </c>
       <c r="J7" s="72">
         <f>I7</f>
@@ -8517,13 +8517,13 @@
         <v/>
       </c>
       <c r="G15" s="77" t="n">
-        <v>226648.4</v>
+        <v>228518.7</v>
       </c>
       <c r="H15" s="77" t="n">
-        <v>203223.3</v>
+        <v>201867.5</v>
       </c>
       <c r="I15" s="77" t="n">
-        <v>203039.7</v>
+        <v>201568</v>
       </c>
       <c r="J15" s="78">
         <f>I15*(1+J7)</f>
@@ -8551,27 +8551,27 @@
       </c>
       <c r="G16" s="82" t="inlineStr">
         <is>
-          <t>194,990 — 261,147</t>
+          <t>196,563 — 263,254</t>
         </is>
       </c>
       <c r="H16" s="82" t="inlineStr">
         <is>
-          <t>184,811 — 216,621</t>
+          <t>183,578 — 215,175</t>
         </is>
       </c>
       <c r="I16" s="82" t="inlineStr">
         <is>
-          <t>202,868 — 203,211</t>
+          <t>199,812 — 203,324</t>
         </is>
       </c>
       <c r="J16" s="82" t="inlineStr">
         <is>
-          <t>204,329 — 267,341</t>
+          <t>187,353 — 245,735</t>
         </is>
       </c>
       <c r="K16" s="82" t="inlineStr">
         <is>
-          <t>204,495 — 267,559</t>
+          <t>187,369 — 245,755</t>
         </is>
       </c>
       <c r="L16" s="83" t="inlineStr">
@@ -8715,13 +8715,13 @@
         <v/>
       </c>
       <c r="G20" s="77" t="n">
-        <v>56273.8</v>
+        <v>56738.1</v>
       </c>
       <c r="H20" s="77" t="n">
-        <v>50457.6</v>
+        <v>50121</v>
       </c>
       <c r="I20" s="77" t="n">
-        <v>50412</v>
+        <v>50046.6</v>
       </c>
       <c r="J20" s="78">
         <f>J15*J8</f>
@@ -8749,27 +8749,27 @@
       </c>
       <c r="G21" s="82" t="inlineStr">
         <is>
-          <t>48,413 — 64,839</t>
+          <t>48,804 — 65,362</t>
         </is>
       </c>
       <c r="H21" s="82" t="inlineStr">
         <is>
-          <t>45,886 — 53,784</t>
+          <t>45,580 — 53,425</t>
         </is>
       </c>
       <c r="I21" s="82" t="inlineStr">
         <is>
-          <t>50,369 — 50,455</t>
+          <t>49,611 — 50,483</t>
         </is>
       </c>
       <c r="J21" s="82" t="inlineStr">
         <is>
-          <t>50,732 — 66,377</t>
+          <t>46,517 — 61,013</t>
         </is>
       </c>
       <c r="K21" s="82" t="inlineStr">
         <is>
-          <t>50,773 — 66,431</t>
+          <t>46,521 — 61,018</t>
         </is>
       </c>
       <c r="L21" s="83" t="inlineStr">
@@ -9422,7 +9422,7 @@
       <c r="L37" s="99" t="n"/>
       <c r="M37" s="74" t="inlineStr">
         <is>
-          <t>Growth tier: LOW (-7.6% 3yr avg rev growth).  Bear 2.00% / Base 2.5% / Bull 3.00%.  Keep below WACC.</t>
+          <t>Growth tier: LOW (-3.2% 3yr avg rev growth).  Bear 2.00% / Base 2.5% / Bull 3.00%.  Keep below WACC.</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9447,7 @@
       <c r="L38" s="99" t="n"/>
       <c r="M38" s="74" t="inlineStr">
         <is>
-          <t>Growth tier: LOW (-7.6% 3yr avg rev growth).  Bear 8x / Base 10x / Bull 12x.  Override manually if needed.</t>
+          <t>Growth tier: LOW (-3.2% 3yr avg rev growth).  Bear 8x / Base 10x / Bull 12x.  Override manually if needed.</t>
         </is>
       </c>
     </row>
@@ -9949,7 +9949,7 @@
         </is>
       </c>
       <c r="B61" s="112" t="n">
-        <v>186.6</v>
+        <v>191.43</v>
       </c>
       <c r="C61" s="104" t="n"/>
       <c r="D61" s="104" t="n"/>
@@ -10049,7 +10049,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="114" t="inlineStr">
         <is>
-          <t>JS SCORECARD — CVX  |  Master Prompt v2  |  15 May 2026  |  Sector bucket: Cyclical</t>
+          <t>JS SCORECARD — CVX  |  Master Prompt v2  |  24 May 2026  |  Sector bucket: Cyclical</t>
         </is>
       </c>
     </row>
@@ -10182,7 +10182,7 @@
       </c>
       <c r="D9" s="130" t="inlineStr">
         <is>
-          <t>GM 30.4% ✗ (&gt;40%)  |  GM trend +2.6% ✓ (&gt;+1pp)  |  ROIC-WACC +2.4% ✗ (&gt;+5pp)  |  Rev consistency σ=26.2% ✗ (&lt;8%)  [1/4 indicators positive — proxy score]</t>
+          <t>GM 30.4% ✗ (&gt;40%)  |  GM trend +2.6% ✓ (&gt;+1pp)  |  ROIC-WACC -1.4% ✗ (&gt;+5pp)  |  Rev consistency σ=26.2% ✗ (&lt;8%)  [1/4 indicators positive — proxy score]</t>
         </is>
       </c>
       <c r="E9" s="131" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="H9" s="134" t="inlineStr">
         <is>
-          <t>GM 30.4% ✗ (&gt;40%)  |  GM trend +2.6% ✓ (&gt;+1pp)  |  ROIC-WACC +2.4% ✗ (&gt;+5pp)  |  Rev consistency σ=26.2% ✗ (&lt;8%)  [1/4 indicators positive — proxy score]</t>
+          <t>GM 30.4% ✗ (&gt;40%)  |  GM trend +2.6% ✓ (&gt;+1pp)  |  ROIC-WACC -1.4% ✗ (&gt;+5pp)  |  Rev consistency σ=26.2% ✗ (&lt;8%)  [1/4 indicators positive — proxy score]</t>
         </is>
       </c>
     </row>
@@ -10249,7 +10249,7 @@
       </c>
       <c r="D11" s="130" t="inlineStr">
         <is>
-          <t>ROIC trend -12.7% ✗ (≥-2pp)  |  GM maintained +2.6% ✓  |  Op margin -7.9% ✗ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -0.9%/yr ✓ (net buyback)  |  Goodwill/Equity 2% ✓ (&lt;40%)  [3/6 indicators positive — proxy score]</t>
+          <t>ROIC trend -12.7% ✗ (&gt;=-2pp)  |  GM maintained +2.6% ✓  |  Op margin -7.9% ✗ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -0.9%/yr ✓ (net buyback)  |  Goodwill/Equity 2% ✓ (&lt;40%)  [3/6 indicators positive — proxy score]</t>
         </is>
       </c>
       <c r="E11" s="135" t="inlineStr">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="H11" s="134" t="inlineStr">
         <is>
-          <t>ROIC trend -12.7% ✗ (≥-2pp)  |  GM maintained +2.6% ✓  |  Op margin -7.9% ✗ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -0.9%/yr ✓ (net buyback)  |  Goodwill/Equity 2% ✓ (&lt;40%)  [3/6 indicators positive — proxy score]</t>
+          <t>ROIC trend -12.7% ✗ (&gt;=-2pp)  |  GM maintained +2.6% ✓  |  Op margin -7.9% ✗ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -0.9%/yr ✓ (net buyback)  |  Goodwill/Equity 2% ✓ (&lt;40%)  [3/6 indicators positive — proxy score]</t>
         </is>
       </c>
     </row>
@@ -10339,7 +10339,7 @@
         </is>
       </c>
       <c r="F14" s="132" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G14" s="133">
         <f>IF(F14="",0,C14*F14*10)</f>
@@ -10457,7 +10457,7 @@
         </is>
       </c>
       <c r="F18" s="132" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G18" s="133">
         <f>IF(F18="",0,C18*F18*10)</f>
@@ -10494,7 +10494,7 @@
         </is>
       </c>
       <c r="F19" s="132" t="n">
-        <v>11.85</v>
+        <v>10</v>
       </c>
       <c r="G19" s="133">
         <f>IF(F19="",0,C19*F19*10)</f>
@@ -10522,7 +10522,7 @@
       </c>
       <c r="D20" s="130" t="inlineStr">
         <is>
-          <t>Rev growth σ=26.2%  |  Op margin σ=3.4%  [proxy — lower σ = lower risk = higher score]</t>
+          <t>Rev growth σ=26.2%  |  OM trend -1.3%, σ=3.4%  [quality = direction + stability]</t>
         </is>
       </c>
       <c r="E20" s="135" t="inlineStr">
@@ -10539,7 +10539,7 @@
       </c>
       <c r="H20" s="134" t="inlineStr">
         <is>
-          <t>Rev growth σ=26.2%  |  Op margin σ=3.4%  [proxy — lower σ = lower risk = higher score]</t>
+          <t>Rev growth σ=26.2%  |  OM trend -1.3%, σ=3.4%  [quality = direction + stability]</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="D22" s="130" t="inlineStr">
         <is>
-          <t>Current 22.9x  |  5yr avg 15.0x  |  DCF-implied 36.1x  [+53% vs benchmark]</t>
+          <t>Current 22.9x  |  5yr avg 15.0x  |  DCF-implied 26.3x [ref only — not used as benchmark]  [+53% vs benchmark]  [trail=0.00 | fwd_pe=14.1x→7.90 | abs=7.0 → blended 40/40/20=4.56]  PEG=13.56 (fwd_pe=14.1x / eps_growth=104%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
       <c r="E22" s="131" t="inlineStr">
@@ -10575,7 +10575,7 @@
         </is>
       </c>
       <c r="F22" s="132" t="n">
-        <v>0</v>
+        <v>5.06</v>
       </c>
       <c r="G22" s="133">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10583,7 +10583,7 @@
       </c>
       <c r="H22" s="134" t="inlineStr">
         <is>
-          <t>Current 22.9x  |  5yr avg 15.0x  |  DCF-implied 36.1x  [+53% vs benchmark]</t>
+          <t>Current 22.9x  |  5yr avg 15.0x  |  DCF-implied 26.3x [ref only — not used as benchmark]  [+53% vs benchmark]  [trail=0.00 | fwd_pe=14.1x→7.90 | abs=7.0 → blended 40/40/20=4.56]  PEG=13.56 (fwd_pe=14.1x / eps_growth=104%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="D23" s="130" t="inlineStr">
         <is>
-          <t>Current 17.0x  |  5yr avg 13.7x  |  DCF-implied 26.8x  [+24% vs benchmark]</t>
+          <t>Current 17.0x  |  5yr avg 13.7x  |  DCF-implied 19.5x [ref only — not used as benchmark]  [+24% vs benchmark]  [trail=3.15 | fwd_pfcf=17.2x→2.93 | abs=10.0 → blended 40/40/20=4.43]</t>
         </is>
       </c>
       <c r="E23" s="135" t="inlineStr">
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="F23" s="132" t="n">
-        <v>3.15</v>
+        <v>4.43</v>
       </c>
       <c r="G23" s="133">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10620,7 +10620,7 @@
       </c>
       <c r="H23" s="134" t="inlineStr">
         <is>
-          <t>Current 17.0x  |  5yr avg 13.7x  |  DCF-implied 26.8x  [+24% vs benchmark]</t>
+          <t>Current 17.0x  |  5yr avg 13.7x  |  DCF-implied 19.5x [ref only — not used as benchmark]  [+24% vs benchmark]  [trail=3.15 | fwd_pfcf=17.2x→2.93 | abs=10.0 → blended 40/40/20=4.43]</t>
         </is>
       </c>
     </row>

</xml_diff>